<commit_message>
IKA Toplu Update via Panel
</commit_message>
<xml_diff>
--- a/THA.xlsx
+++ b/THA.xlsx
@@ -474,7 +474,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>Gönderildi</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>Evet</v>
       </c>
       <c r="N2" t="str">
         <v/>

</xml_diff>